<commit_message>
Financial Model Draft added
</commit_message>
<xml_diff>
--- a/Financial Projections/Financial Projections.xlsx
+++ b/Financial Projections/Financial Projections.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cwbec\BlockMed\BlockMed\Financial Projections\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54C5B9F5-F7D7-4454-BAAD-30E68F7793F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B99F7EB-9008-432E-BD5F-4AB1E8D1A613}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12710" yWindow="0" windowWidth="12980" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Samp" sheetId="6" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="Rev Timeline" sheetId="3" r:id="rId4"/>
     <sheet name="Cost Timeline" sheetId="4" r:id="rId5"/>
     <sheet name="HR" sheetId="5" r:id="rId6"/>
+    <sheet name="Equity" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="53">
   <si>
     <t>Active Customers (EOY)</t>
   </si>
@@ -107,6 +108,99 @@
   </si>
   <si>
     <t>year 3</t>
+  </si>
+  <si>
+    <t>Initial Inv</t>
+  </si>
+  <si>
+    <t>minimum pay</t>
+  </si>
+  <si>
+    <t>Dan</t>
+  </si>
+  <si>
+    <t>Reshi</t>
+  </si>
+  <si>
+    <t>Nick</t>
+  </si>
+  <si>
+    <t>Bhadri</t>
+  </si>
+  <si>
+    <t>Tamer</t>
+  </si>
+  <si>
+    <t>Conrad</t>
+  </si>
+  <si>
+    <t>Equity Ask</t>
+  </si>
+  <si>
+    <t>Angel Investors</t>
+  </si>
+  <si>
+    <t>Customer acquisition (EOY): 20 (Y1) → 110 (Y2) → 350 (Y3)</t>
+  </si>
+  <si>
+    <t>- Deals per customer per year: 1.5–2.5 (Y1, ramp) → 3 (Y2) → 3.5 (Y3, repeats compound)</t>
+  </si>
+  <si>
+    <t>- Avg ticket size: $25K (Y1) → $35K (Y2) → $50K (Y3)</t>
+  </si>
+  <si>
+    <t>- Blended settlement-fee take rate: 0.7% per trade (range across tiers)</t>
+  </si>
+  <si>
+    <t>- Tier mix (Tier A eBL / Tier C paper): 30 / 70 (Y1) → 50 / 50 (Y2) → 60 / 40 (Y3)</t>
+  </si>
+  <si>
+    <t>- Headcount: 6 founders (Y1) → 8 (Y2) → 12 (Y3)</t>
+  </si>
+  <si>
+    <t>- Founder salaries: $20K Y1 (equity-heavy) → $45K Y2 → $55K Y3</t>
+  </si>
+  <si>
+    <t>- SaaS Stream B requires 1 partner in Y1, 2–3 in Y2, 4–5 in Y3</t>
+  </si>
+  <si>
+    <t>- Yield share Stream C depends on regulated yield infrastructure becoming available</t>
+  </si>
+  <si>
+    <t>deals per customer per year</t>
+  </si>
+  <si>
+    <t>low</t>
+  </si>
+  <si>
+    <t>high</t>
+  </si>
+  <si>
+    <t>avg ticket size</t>
+  </si>
+  <si>
+    <t>yr 2</t>
+  </si>
+  <si>
+    <t>yr 3</t>
+  </si>
+  <si>
+    <t>settlement fee take rate</t>
+  </si>
+  <si>
+    <t>tier Mix</t>
+  </si>
+  <si>
+    <t>Headcount</t>
+  </si>
+  <si>
+    <t>Founder Salaries</t>
+  </si>
+  <si>
+    <t>Saas Stream B</t>
+  </si>
+  <si>
+    <t>Yield Share</t>
   </si>
 </sst>
 </file>
@@ -117,7 +211,7 @@
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="166" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -131,6 +225,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="7"/>
+      <color rgb="FF000000"/>
+      <name val="Courier New"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -154,10 +254,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -439,10 +545,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F4273C1-009D-4CD2-86ED-4FF4719728EC}">
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="65.08984375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20.453125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -479,24 +585,32 @@
         <f>(25+55)/2</f>
         <v>40</v>
       </c>
+      <c r="C3">
+        <v>300</v>
+      </c>
+      <c r="D3">
+        <v>1200</v>
+      </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>14</v>
       </c>
       <c r="B4">
-        <f t="shared" ref="B4:B7" si="0">(25+55)/2</f>
-        <v>40</v>
+        <f>25000</f>
+        <v>25000</v>
+      </c>
+      <c r="C4">
+        <v>35000</v>
+      </c>
+      <c r="D4">
+        <v>50000</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>15</v>
       </c>
-      <c r="B5">
-        <f>(5+35)/2</f>
-        <v>20</v>
-      </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
@@ -506,13 +620,27 @@
         <f>(155+260)/2</f>
         <v>207.5</v>
       </c>
+      <c r="C6">
+        <f>(475000+735000)/2</f>
+        <v>605000</v>
+      </c>
+      <c r="D6">
+        <f>(1100000+1700000)/2</f>
+        <v>1400000</v>
+      </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="2">
+      <c r="B7" s="3">
         <v>0.65</v>
+      </c>
+      <c r="C7" s="3">
+        <v>0.65</v>
+      </c>
+      <c r="D7" s="3">
+        <v>0.7</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
@@ -524,7 +652,7 @@
       <c r="A10" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="1">
+      <c r="B10" s="2">
         <v>2500000000000</v>
       </c>
     </row>
@@ -532,7 +660,7 @@
       <c r="A11" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="1">
+      <c r="B11" s="2">
         <v>5000000000</v>
       </c>
     </row>
@@ -540,8 +668,155 @@
       <c r="A12" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="1">
+      <c r="B12" s="2">
         <v>250000000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A18" s="5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A19" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20" s="5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21" s="5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A22" s="5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A23" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B25" t="s">
+        <v>42</v>
+      </c>
+      <c r="C25" t="s">
+        <v>43</v>
+      </c>
+      <c r="D25" t="s">
+        <v>45</v>
+      </c>
+      <c r="E25" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A26" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B26">
+        <v>1.5</v>
+      </c>
+      <c r="C26">
+        <v>2.5</v>
+      </c>
+      <c r="D26">
+        <v>3</v>
+      </c>
+      <c r="E26">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A27" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B27">
+        <v>25000</v>
+      </c>
+      <c r="D27">
+        <v>35000</v>
+      </c>
+      <c r="E27">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A28" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B28" s="6">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="D28" s="6">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="E28" s="6">
+        <v>7.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A29" s="5" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A31" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="B31">
+        <v>6</v>
+      </c>
+      <c r="D31">
+        <v>8</v>
+      </c>
+      <c r="E31">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A32" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="B32">
+        <v>20000</v>
+      </c>
+      <c r="D32">
+        <v>45000</v>
+      </c>
+      <c r="E32">
+        <v>55000</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A33" s="5" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A34" s="5" t="s">
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -551,9 +826,21 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55174C66-08CC-4C33-84B2-7EA2B723F292}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="13.6328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" s="1">
+        <v>1000000</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -651,6 +938,115 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A75885B-C936-48F8-A5C6-3779982D82C3}">
+  <dimension ref="A1:F10"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="13.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.26953125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" s="3">
+        <v>0.2</v>
+      </c>
+      <c r="E1" s="3">
+        <v>0.8</v>
+      </c>
+      <c r="F1">
+        <f>80/6</f>
+        <v>13.333333333333334</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="B2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3" s="3">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4">
+        <v>18000</v>
+      </c>
+      <c r="C4" s="3">
+        <v>0.17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6">
+        <v>30000</v>
+      </c>
+      <c r="C6" s="3">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" s="4">
+        <v>80000</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E9" s="3">
+        <f>E1-SUM(C3:C8)</f>
+        <v>0.43000000000000005</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="B10">
+        <f>SUM(B3:B8)</f>
+        <v>188000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C608D163-8B6B-4DB5-B230-4C38BE78B5EE}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData/>

</xml_diff>